<commit_message>
feat: nota; update: tambahkan kolom pph21 ke upload gaji
</commit_message>
<xml_diff>
--- a/assets/template_upload_gajian_monthly.xlsx
+++ b/assets/template_upload_gajian_monthly.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\bariskode\upload\hris\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\bariskode\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C493B2E2-CCDD-4CC8-82A8-8E18DE82935C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69945FF-E250-4D3C-BF99-0DDAEE2BEC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{54297741-F157-49E4-BB90-3AACE9B6041D}"/>
   </bookViews>
@@ -129,13 +129,13 @@
     <t>tgl_gaji</t>
   </si>
   <si>
-    <t>Pot. Parkir</t>
-  </si>
-  <si>
     <t>Nama Staff</t>
   </si>
   <si>
     <t>Jabatan staff</t>
+  </si>
+  <si>
+    <t>PPH21</t>
   </si>
 </sst>
 </file>
@@ -173,14 +173,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -332,22 +333,22 @@
     <xf numFmtId="167" fontId="2" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -777,20 +778,20 @@
       <c r="AA1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="11" t="s">
+      <c r="AB1" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="11" t="s">
+      <c r="AC1" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="12" t="s">
+      <c r="AD1" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="13" t="s">
+      <c r="AE1" s="17" t="s">
         <v>30</v>
       </c>
       <c r="AF1" s="14" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -798,12 +799,12 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
         <v>32</v>
       </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" s="16">
+      <c r="D2" s="12">
         <v>45293</v>
       </c>
       <c r="E2">
@@ -881,10 +882,10 @@
       <c r="AC2">
         <v>0</v>
       </c>
-      <c r="AD2" s="17">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="15">
+      <c r="AD2" s="13">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="11">
         <v>45681</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update: header row excel upload gaji
</commit_message>
<xml_diff>
--- a/assets/template_upload_gajian_monthly.xlsx
+++ b/assets/template_upload_gajian_monthly.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\bariskode\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69945FF-E250-4D3C-BF99-0DDAEE2BEC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB48E83-0186-4221-B976-FB69ED3A0557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{54297741-F157-49E4-BB90-3AACE9B6041D}"/>
   </bookViews>
@@ -688,12 +688,12 @@
     <col min="20" max="20" width="9.109375" customWidth="1"/>
     <col min="21" max="22" width="10.88671875" customWidth="1"/>
     <col min="23" max="23" width="9.109375" customWidth="1"/>
-    <col min="24" max="24" width="10.88671875" customWidth="1"/>
-    <col min="25" max="25" width="13.44140625" customWidth="1"/>
-    <col min="26" max="26" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="27" max="29" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.88671875" customWidth="1"/>
+    <col min="26" max="26" width="13.44140625" customWidth="1"/>
+    <col min="27" max="27" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="30" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="10" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="55.2" x14ac:dyDescent="0.3">
@@ -766,32 +766,32 @@
       <c r="W1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="X1" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="8" t="s">
+      <c r="Z1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="AA1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="10" t="s">
+      <c r="AB1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="15" t="s">
+      <c r="AC1" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="15" t="s">
+      <c r="AD1" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="16" t="s">
+      <c r="AE1" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="17" t="s">
+      <c r="AF1" s="17" t="s">
         <v>30</v>
-      </c>
-      <c r="AF1" s="14" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -864,9 +864,6 @@
       <c r="W2">
         <v>0</v>
       </c>
-      <c r="X2">
-        <v>0</v>
-      </c>
       <c r="Y2">
         <v>0</v>
       </c>
@@ -882,10 +879,13 @@
       <c r="AC2">
         <v>0</v>
       </c>
-      <c r="AD2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="11">
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="13">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="11">
         <v>45681</v>
       </c>
     </row>

</xml_diff>